<commit_message>
Add BIP-39 flashcard images and update generation status
</commit_message>
<xml_diff>
--- a/bip-39-words.xlsx
+++ b/bip-39-words.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zubinpijit/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zubinpijit/bithope-ops/hobbyprojects/bitcointetris/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8C1B2E8-CE62-1541-95E7-F1870FB1BE92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DC3A67-DABA-2D4D-88E1-024EBD125295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{BB049F76-9FC2-F643-AF95-02F941E60D0C}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="17040" activeTab="1" xr2:uid="{BB049F76-9FC2-F643-AF95-02F941E60D0C}"/>
   </bookViews>
   <sheets>
     <sheet name="wordlist" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1616" uniqueCount="963">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1616" uniqueCount="964">
   <si>
     <t>ลำดับ (Index)</t>
   </si>
@@ -2927,6 +2927,9 @@
   </si>
   <si>
     <t xml:space="preserve">ฉันต้องการสร้างภาพประกอบคำศัพท์ BIP-39 สำหรับเด็กและผู้เริ่มเรียนรู้ภาษาอังกฤษ เป้าหมาย: สร้างภาพประกอบแบบ flashcard ทีละคำ สำหรับคำศัพท์ 4 ตัวอักษรจาก BIP-39 wordlist เพื่อใช้ทำฐานข้อมูลการเรียนรู้คำศัพท์ สไตล์ภาพที่ต้องการ: * ภาพเดี่ยว 1 คำต่อ 1 รูป * ขนาดสี่เหลี่ยมจัตุรัส 1:1 * พื้นหลังสีขาวหรือ off-white สะอาด * ภาพวาดการ์ตูน 2D / soft vector illustration * โทนสดใส เป็นมิตรกับเด็ก * เส้นขอบนุ่ม สะอาด ไม่รก * แสงเงานุ่ม ๆ คล้าย educational flashcard * วัตถุหลักอยู่กึ่งกลางภาพ * มีคำศัพท์ภาษาอังกฤษตัวพิมพ์เล็กอยู่ด้านล่างภาพ * ฟอนต์ควรดูมน อ่านง่าย สีกรมท่าหรือสีเข้ม * หลีกเลี่ยงภาพเหมือนจริง ภาพซับซ้อน หรือฉากหลังเยอะ * หลีกเลี่ยงการทำเป็นตารางรวมหลายคำ * ห้ามรวมหลายคำในภาพเดียว * ห้ามใส่คำแปลภาษาไทยในภาพ * ห้ามใส่หัวตาราง คอลัมน์ หรือ layout แบบ spreadsheet ตัวอย่าง tone ที่ต้องการ: ภาพคำว่า able = เด็กยิ้มยกนิ้วโป้ง พร้อมคำว่า “able” ด้านล่าง คำสั่งสำคัญ: ให้สร้างภาพแยกทีละคำเท่านั้น ไม่ใช่ infographic ไม่ใช่ตาราง ไม่ใช่ collage ถ้าสร้างหลายภาพใน batch เดียว ให้แต่ละภาพเป็น flashcard เดี่ยวแยกกัน ทุกภาพต้องมี style เดียวกันกับตัวอย่างด้านบน รายการคำที่จะสร้างใน batch นี้  และ concept ภาพ จะแนบมา Output ที่ต้องการ: สร้างภาพ flashcard เดี่ยว 1 รูปต่อ 1 คำ ตาม style เดียวกันทั้งหมด ขนาด 1024x1024 px พร้อมทั้งตั้งชื่อไฟล์ตามชื่อ word นั้น เช่น blur.png เป็นต้น </t>
+  </si>
+  <si>
+    <t>คนนั่งสมาธิยิ้มสงบ</t>
   </si>
 </sst>
 </file>
@@ -2961,7 +2964,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2971,12 +2974,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3010,7 +3007,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
@@ -8839,7 +8836,9 @@
   <cols>
     <col min="1" max="3" width="10.7109375" style="5"/>
     <col min="4" max="4" width="10.7109375" style="4"/>
-    <col min="5" max="16384" width="10.7109375" style="5"/>
+    <col min="5" max="5" width="10.7109375" style="5"/>
+    <col min="6" max="6" width="19.42578125" style="5" customWidth="1"/>
+    <col min="7" max="16384" width="10.7109375" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="4:6" x14ac:dyDescent="0.45">
@@ -9352,7 +9351,7 @@
       <c r="D47" s="4">
         <v>46</v>
       </c>
-      <c r="E47" s="7" t="s">
+      <c r="E47" s="5" t="s">
         <v>138</v>
       </c>
       <c r="F47" s="5" t="s">
@@ -9363,7 +9362,7 @@
       <c r="D48" s="4">
         <v>47</v>
       </c>
-      <c r="E48" s="8" t="s">
+      <c r="E48" s="5" t="s">
         <v>141</v>
       </c>
       <c r="F48" s="5" t="s">
@@ -9374,7 +9373,7 @@
       <c r="D49" s="4">
         <v>48</v>
       </c>
-      <c r="E49" s="8" t="s">
+      <c r="E49" s="5" t="s">
         <v>144</v>
       </c>
       <c r="F49" s="5" t="s">
@@ -9385,18 +9384,18 @@
       <c r="D50" s="4">
         <v>49</v>
       </c>
-      <c r="E50" s="8" t="s">
+      <c r="E50" s="5" t="s">
         <v>147</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>149</v>
+        <v>963</v>
       </c>
     </row>
     <row r="51" spans="4:8" x14ac:dyDescent="0.45">
       <c r="D51" s="4">
         <v>50</v>
       </c>
-      <c r="E51" s="8" t="s">
+      <c r="E51" s="5" t="s">
         <v>150</v>
       </c>
       <c r="F51" s="5" t="s">
@@ -9454,7 +9453,7 @@
       <c r="D56" s="4">
         <v>55</v>
       </c>
-      <c r="E56" s="5" t="s">
+      <c r="E56" s="8" t="s">
         <v>165</v>
       </c>
       <c r="F56" s="5" t="s">
@@ -9509,7 +9508,7 @@
       <c r="D61" s="4">
         <v>60</v>
       </c>
-      <c r="E61" s="5" t="s">
+      <c r="E61" s="7" t="s">
         <v>180</v>
       </c>
       <c r="F61" s="5" t="s">

</xml_diff>